<commit_message>
Implemented confidence scoring, end-to-end hybrid
</commit_message>
<xml_diff>
--- a/docs/Updated Gantt Chart.xlsx
+++ b/docs/Updated Gantt Chart.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aryan\Disseratation\intelligent-guitar-practice\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{999AAF89-78C3-4AB3-B57B-4F26C5F5BCEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F04937D-153B-4943-9E79-F645CF9AF723}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" xr2:uid="{C592EF48-8C9B-48D2-B5FD-A85F508DB3A8}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="91">
   <si>
     <t>Task</t>
   </si>
@@ -150,9 +150,6 @@
     <t>Improve Tab Generation (Chords, Polyphonic Audio)</t>
   </si>
   <si>
-    <t>Automatic Audio Segmentation Implementation</t>
-  </si>
-  <si>
     <t>Mar W1</t>
   </si>
   <si>
@@ -165,9 +162,6 @@
     <t>2 weeks</t>
   </si>
   <si>
-    <t>User Testing &amp; Evaluation Study</t>
-  </si>
-  <si>
     <t>Apr W3</t>
   </si>
   <si>
@@ -243,9 +237,6 @@
     <t>Nov W1</t>
   </si>
   <si>
-    <t>Guitar Technique Classification</t>
-  </si>
-  <si>
     <t>Multi Track Audio Separation</t>
   </si>
   <si>
@@ -286,9 +277,6 @@
   </si>
   <si>
     <t>Nov W3</t>
-  </si>
-  <si>
-    <t>Feb W1</t>
   </si>
   <si>
     <t>6 weeks</t>
@@ -354,13 +342,22 @@
     </r>
   </si>
   <si>
-    <t>Dec W3</t>
-  </si>
-  <si>
     <t>Jan W2</t>
   </si>
   <si>
-    <t>Feb W4</t>
+    <t>Traffic Confidence Score System</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Audio Player and MIDI Player </t>
+  </si>
+  <si>
+    <t>Qualitative Evaluation</t>
+  </si>
+  <si>
+    <t>Feb W2</t>
+  </si>
+  <si>
+    <t>Feb W3</t>
   </si>
 </sst>
 </file>
@@ -793,7 +790,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -869,18 +866,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
@@ -895,6 +880,22 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1241,70 +1242,70 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" x14ac:dyDescent="0.3">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="56" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="41" t="s">
+      <c r="B1" s="55" t="s">
         <v>10</v>
       </c>
-      <c r="C1" s="39" t="s">
+      <c r="C1" s="53" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="39"/>
-      <c r="E1" s="39"/>
-      <c r="F1" s="39"/>
-      <c r="G1" s="39" t="s">
+      <c r="D1" s="53"/>
+      <c r="E1" s="53"/>
+      <c r="F1" s="53"/>
+      <c r="G1" s="53" t="s">
         <v>2</v>
       </c>
-      <c r="H1" s="39"/>
-      <c r="I1" s="39"/>
-      <c r="J1" s="39"/>
-      <c r="K1" s="39" t="s">
+      <c r="H1" s="53"/>
+      <c r="I1" s="53"/>
+      <c r="J1" s="53"/>
+      <c r="K1" s="53" t="s">
         <v>3</v>
       </c>
-      <c r="L1" s="39"/>
-      <c r="M1" s="39"/>
-      <c r="N1" s="39"/>
-      <c r="O1" s="39" t="s">
+      <c r="L1" s="53"/>
+      <c r="M1" s="53"/>
+      <c r="N1" s="53"/>
+      <c r="O1" s="53" t="s">
         <v>4</v>
       </c>
-      <c r="P1" s="39"/>
-      <c r="Q1" s="39"/>
-      <c r="R1" s="39"/>
-      <c r="S1" s="39" t="s">
+      <c r="P1" s="53"/>
+      <c r="Q1" s="53"/>
+      <c r="R1" s="53"/>
+      <c r="S1" s="53" t="s">
         <v>5</v>
       </c>
-      <c r="T1" s="39"/>
-      <c r="U1" s="39"/>
-      <c r="V1" s="39"/>
-      <c r="W1" s="39" t="s">
+      <c r="T1" s="53"/>
+      <c r="U1" s="53"/>
+      <c r="V1" s="53"/>
+      <c r="W1" s="53" t="s">
         <v>6</v>
       </c>
-      <c r="X1" s="39"/>
-      <c r="Y1" s="39"/>
-      <c r="Z1" s="39"/>
-      <c r="AA1" s="39" t="s">
+      <c r="X1" s="53"/>
+      <c r="Y1" s="53"/>
+      <c r="Z1" s="53"/>
+      <c r="AA1" s="53" t="s">
         <v>7</v>
       </c>
-      <c r="AB1" s="39"/>
-      <c r="AC1" s="39"/>
-      <c r="AD1" s="39"/>
-      <c r="AE1" s="39" t="s">
+      <c r="AB1" s="53"/>
+      <c r="AC1" s="53"/>
+      <c r="AD1" s="53"/>
+      <c r="AE1" s="53" t="s">
         <v>8</v>
       </c>
-      <c r="AF1" s="39"/>
-      <c r="AG1" s="39"/>
-      <c r="AH1" s="39"/>
-      <c r="AI1" s="39" t="s">
+      <c r="AF1" s="53"/>
+      <c r="AG1" s="53"/>
+      <c r="AH1" s="53"/>
+      <c r="AI1" s="53" t="s">
         <v>9</v>
       </c>
-      <c r="AJ1" s="39"/>
-      <c r="AK1" s="39"/>
-      <c r="AL1" s="40"/>
+      <c r="AJ1" s="53"/>
+      <c r="AK1" s="53"/>
+      <c r="AL1" s="54"/>
     </row>
     <row r="2" spans="1:38" x14ac:dyDescent="0.3">
-      <c r="A2" s="42"/>
-      <c r="B2" s="41"/>
+      <c r="A2" s="56"/>
+      <c r="B2" s="55"/>
       <c r="C2" s="2">
         <v>1</v>
       </c>
@@ -1680,7 +1681,7 @@
     </row>
     <row r="9" spans="1:38" x14ac:dyDescent="0.3">
       <c r="A9" s="11" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="B9" s="4">
         <v>5</v>
@@ -1870,18 +1871,18 @@
       <c r="J13" s="2"/>
       <c r="K13" s="2"/>
       <c r="L13" s="2"/>
-      <c r="M13" s="23"/>
-      <c r="N13" s="23"/>
-      <c r="O13" s="23"/>
+      <c r="M13" s="2"/>
+      <c r="N13" s="2"/>
+      <c r="O13" s="2"/>
       <c r="P13" s="23"/>
       <c r="Q13" s="5"/>
       <c r="R13" s="5"/>
-      <c r="S13" s="2"/>
-      <c r="T13" s="2"/>
-      <c r="U13" s="2"/>
-      <c r="V13" s="2"/>
-      <c r="W13" s="2"/>
-      <c r="X13" s="2"/>
+      <c r="S13" s="23"/>
+      <c r="T13" s="23"/>
+      <c r="U13" s="23"/>
+      <c r="V13" s="23"/>
+      <c r="W13" s="23"/>
+      <c r="X13" s="23"/>
       <c r="Y13" s="2"/>
       <c r="Z13" s="2"/>
       <c r="AA13" s="2"/>
@@ -1917,10 +1918,10 @@
       <c r="M14" s="2"/>
       <c r="N14" s="2"/>
       <c r="O14" s="2"/>
-      <c r="P14" s="23"/>
+      <c r="P14" s="58"/>
       <c r="Q14" s="5"/>
       <c r="R14" s="5"/>
-      <c r="S14" s="23"/>
+      <c r="S14" s="58"/>
       <c r="T14" s="23"/>
       <c r="U14" s="23"/>
       <c r="V14" s="2"/>
@@ -1931,9 +1932,9 @@
       <c r="AA14" s="2"/>
       <c r="AB14" s="2"/>
       <c r="AC14" s="2"/>
-      <c r="AD14" s="48"/>
-      <c r="AE14" s="49"/>
-      <c r="AF14" s="50"/>
+      <c r="AD14" s="44"/>
+      <c r="AE14" s="45"/>
+      <c r="AF14" s="46"/>
       <c r="AG14" s="5"/>
       <c r="AH14" s="5"/>
       <c r="AI14" s="5"/>
@@ -1961,13 +1962,13 @@
       <c r="M15" s="2"/>
       <c r="N15" s="2"/>
       <c r="O15" s="2"/>
-      <c r="P15" s="23"/>
+      <c r="P15" s="58"/>
       <c r="Q15" s="5"/>
       <c r="R15" s="5"/>
-      <c r="S15" s="23"/>
-      <c r="T15" s="23"/>
+      <c r="S15" s="58"/>
+      <c r="T15" s="58"/>
       <c r="U15" s="23"/>
-      <c r="V15" s="2"/>
+      <c r="V15" s="23"/>
       <c r="W15" s="2"/>
       <c r="X15" s="2"/>
       <c r="Y15" s="2"/>
@@ -1975,9 +1976,9 @@
       <c r="AA15" s="2"/>
       <c r="AB15" s="2"/>
       <c r="AC15" s="2"/>
-      <c r="AD15" s="46"/>
-      <c r="AE15" s="52"/>
-      <c r="AF15" s="51"/>
+      <c r="AD15" s="42"/>
+      <c r="AE15" s="48"/>
+      <c r="AF15" s="47"/>
       <c r="AG15" s="5"/>
       <c r="AH15" s="5"/>
       <c r="AI15" s="5"/>
@@ -2008,9 +2009,9 @@
       <c r="P16" s="2"/>
       <c r="Q16" s="5"/>
       <c r="R16" s="5"/>
-      <c r="S16" s="23"/>
-      <c r="T16" s="23"/>
-      <c r="U16" s="23"/>
+      <c r="S16" s="58"/>
+      <c r="T16" s="58"/>
+      <c r="U16" s="58"/>
       <c r="V16" s="23"/>
       <c r="W16" s="2"/>
       <c r="X16" s="2"/>
@@ -2020,9 +2021,9 @@
       <c r="AB16" s="2"/>
       <c r="AC16" s="2"/>
       <c r="AD16" s="2"/>
-      <c r="AE16" s="47"/>
-      <c r="AF16" s="55"/>
-      <c r="AG16" s="56"/>
+      <c r="AE16" s="43"/>
+      <c r="AF16" s="51"/>
+      <c r="AG16" s="52"/>
       <c r="AH16" s="5"/>
       <c r="AI16" s="5"/>
       <c r="AJ16" s="2"/>
@@ -2031,7 +2032,7 @@
     </row>
     <row r="17" spans="1:38" x14ac:dyDescent="0.3">
       <c r="A17" s="11" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B17" s="4">
         <v>3</v>
@@ -2064,9 +2065,9 @@
       <c r="AB17" s="2"/>
       <c r="AC17" s="2"/>
       <c r="AD17" s="2"/>
-      <c r="AE17" s="45"/>
-      <c r="AF17" s="53"/>
-      <c r="AG17" s="54"/>
+      <c r="AE17" s="41"/>
+      <c r="AF17" s="49"/>
+      <c r="AG17" s="50"/>
       <c r="AH17" s="5"/>
       <c r="AI17" s="5"/>
       <c r="AJ17" s="2"/>
@@ -2075,7 +2076,7 @@
     </row>
     <row r="18" spans="1:38" x14ac:dyDescent="0.3">
       <c r="A18" s="11" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="B18" s="4">
         <v>6</v>
@@ -2108,8 +2109,8 @@
       <c r="AB18" s="20"/>
       <c r="AC18" s="2"/>
       <c r="AD18" s="2"/>
-      <c r="AE18" s="43"/>
-      <c r="AF18" s="44"/>
+      <c r="AE18" s="39"/>
+      <c r="AF18" s="40"/>
       <c r="AG18" s="5"/>
       <c r="AH18" s="5"/>
       <c r="AI18" s="5"/>
@@ -2119,7 +2120,7 @@
     </row>
     <row r="19" spans="1:38" x14ac:dyDescent="0.3">
       <c r="A19" s="12" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B19" s="4">
         <v>2</v>
@@ -2148,7 +2149,7 @@
       <c r="X19" s="2"/>
       <c r="Y19" s="37"/>
       <c r="Z19" s="37"/>
-      <c r="AA19" s="2"/>
+      <c r="AA19" s="37"/>
       <c r="AB19" s="2"/>
       <c r="AC19" s="2"/>
       <c r="AD19" s="2"/>
@@ -2163,7 +2164,7 @@
     </row>
     <row r="20" spans="1:38" x14ac:dyDescent="0.3">
       <c r="A20" s="12" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="B20" s="32">
         <v>4</v>
@@ -2207,7 +2208,7 @@
     </row>
     <row r="21" spans="1:38" x14ac:dyDescent="0.3">
       <c r="A21" s="12" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="B21" s="6">
         <v>1</v>
@@ -2271,7 +2272,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97EE9156-BE08-4F70-AD1D-4301D6B6195B}">
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.77734375" style="1" customWidth="1"/>
@@ -2297,10 +2298,10 @@
         <v>10</v>
       </c>
       <c r="G1" s="10" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="H1" s="10" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
@@ -2308,19 +2309,19 @@
         <v>11</v>
       </c>
       <c r="B2" s="27" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C2" s="28" t="s">
         <v>29</v>
       </c>
       <c r="D2" s="28" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E2" s="28" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G2" s="13" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="H2" s="14"/>
     </row>
@@ -2329,7 +2330,7 @@
         <v>12</v>
       </c>
       <c r="B3" s="27" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C3" s="28" t="s">
         <v>31</v>
@@ -2338,10 +2339,10 @@
         <v>31</v>
       </c>
       <c r="E3" s="28" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="G3" s="13" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="H3" s="18"/>
     </row>
@@ -2350,19 +2351,19 @@
         <v>13</v>
       </c>
       <c r="B4" s="27" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C4" s="28" t="s">
         <v>31</v>
       </c>
       <c r="D4" s="28" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="E4" s="28" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G4" s="13" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="H4" s="15"/>
     </row>
@@ -2374,16 +2375,16 @@
         <v>33</v>
       </c>
       <c r="C5" s="28" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="D5" s="28" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="E5" s="28" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="G5" s="19" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="H5" s="16"/>
     </row>
@@ -2392,22 +2393,22 @@
         <v>15</v>
       </c>
       <c r="B6" s="27" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C6" s="29" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D6" s="28" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E6" s="28" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="G6" s="13" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="H6" s="17" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
@@ -2418,13 +2419,13 @@
         <v>36</v>
       </c>
       <c r="C7" s="28" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D7" s="28" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="E7" s="28" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -2435,13 +2436,13 @@
         <v>34</v>
       </c>
       <c r="C8" s="28" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D8" s="28" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="E8" s="28" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
@@ -2449,10 +2450,10 @@
         <v>18</v>
       </c>
       <c r="B9" s="27" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="C9" s="28" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="D9" s="28" t="s">
         <v>32</v>
@@ -2466,13 +2467,13 @@
         <v>19</v>
       </c>
       <c r="B10" s="27" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="C10" s="28" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="D10" s="28" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="E10" s="28" t="s">
         <v>30</v>
@@ -2483,13 +2484,13 @@
         <v>20</v>
       </c>
       <c r="B11" s="27" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="C11" s="31" t="s">
         <v>32</v>
       </c>
       <c r="D11" s="31" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="E11" s="28" t="s">
         <v>35</v>
@@ -2500,13 +2501,13 @@
         <v>21</v>
       </c>
       <c r="B12" s="27" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C12" s="28" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="D12" s="28" t="s">
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="E12" s="28" t="s">
         <v>30</v>
@@ -2517,16 +2518,16 @@
         <v>22</v>
       </c>
       <c r="B13" s="27" t="s">
-        <v>70</v>
+        <v>58</v>
       </c>
       <c r="C13" s="28" t="s">
+        <v>89</v>
+      </c>
+      <c r="D13" s="28" t="s">
         <v>90</v>
       </c>
-      <c r="D13" s="28" t="s">
-        <v>62</v>
-      </c>
       <c r="E13" s="28" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.3">
@@ -2534,13 +2535,13 @@
         <v>23</v>
       </c>
       <c r="B14" s="27" t="s">
-        <v>37</v>
+        <v>86</v>
       </c>
       <c r="C14" s="28" t="s">
         <v>90</v>
       </c>
       <c r="D14" s="28" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E14" s="28" t="s">
         <v>30</v>
@@ -2551,13 +2552,13 @@
         <v>24</v>
       </c>
       <c r="B15" s="27" t="s">
-        <v>60</v>
+        <v>87</v>
       </c>
       <c r="C15" s="28" t="s">
-        <v>83</v>
+        <v>37</v>
       </c>
       <c r="D15" s="28" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E15" s="28" t="s">
         <v>30</v>
@@ -2565,16 +2566,16 @@
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16" s="25" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B16" s="27" t="s">
-        <v>42</v>
+        <v>88</v>
       </c>
       <c r="C16" s="28" t="s">
-        <v>91</v>
+        <v>60</v>
       </c>
       <c r="D16" s="28" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="E16" s="28" t="s">
         <v>35</v>
@@ -2582,74 +2583,74 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" s="25" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="B17" s="27" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C17" s="28" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D17" s="28" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E17" s="28" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" s="25" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B18" s="27" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C18" s="28" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="D18" s="28" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E18" s="28" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" s="25" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="B19" s="27" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C19" s="28" t="s">
+        <v>41</v>
+      </c>
+      <c r="D19" s="28" t="s">
         <v>43</v>
-      </c>
-      <c r="D19" s="28" t="s">
-        <v>45</v>
       </c>
       <c r="E19" s="28" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A20" s="30" t="s">
-        <v>80</v>
+      <c r="A20" s="57" t="s">
+        <v>77</v>
       </c>
       <c r="B20" s="27" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C20" s="28" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D20" s="28" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="E20" s="28" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A23" s="24"/>
+        <v>47</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A25" s="24"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>